<commit_message>
docs: lock seisen IF increment estimate and add furigana talk tracks
Refresh the standard/risk packs after the 9/29 master reuse lock, and add bilingual scripts with kana so the 160.5人日 case can be read aloud.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PMI/Sinops/phase2-detail-design/sources/20260921-生鮮IF増分見積/【見積】生鮮IF増分_リスク込み案_調査Mappingから詳細設計開発単体_20260921.xlsx
+++ b/PMI/Sinops/phase2-detail-design/sources/20260921-生鮮IF増分見積/【見積】生鮮IF増分_リスク込み案_調査Mappingから詳細設計開発単体_20260921.xlsx
@@ -687,7 +687,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>2026/09/21</t>
+          <t>2026/09/30</t>
         </is>
       </c>
       <c r="C3" s="5" t="n"/>
@@ -765,10 +765,10 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>64.5</v>
+        <v>62</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>2580000</v>
+        <v>2480000</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -784,10 +784,10 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>235.5</v>
+        <v>170</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>6476250</v>
+        <v>4675000</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -803,10 +803,10 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>300</v>
+        <v>232</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>9056250</v>
+        <v>7155000</v>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
@@ -822,10 +822,10 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>1200000</v>
+        <v>920000</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="B13" s="15" t="n">
-        <v>330</v>
+        <v>255</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>10256250</v>
+        <v>8075000</v>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">　生鮮専用マスタの新規本数・既存波及が大きい場合の工数　／　単価：Phase1=40,000・Phase2直接=27,500・PJ管理=40,000（円/人日・税抜）</t>
+          <t xml:space="preserve">　流用判定が一部覆る、倉庫商品マスタが要IF、またはS12/S13のSQL／作成時刻が想定より重い場合　／　単価：Phase1=40,000・Phase2直接=27,500・PJ管理=40,000（円/人日・税抜）</t>
         </is>
       </c>
     </row>
@@ -906,18 +906,18 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>先行トラン（新規IF 4本）</t>
+          <t>確定IF（勧告1.5＋変換1＋入荷2＋スケジュール1）</t>
         </is>
       </c>
       <c r="C18" s="19" t="n">
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="D18" s="20" t="n">
-        <v>3606250</v>
+        <v>4590000</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>Phase1 24.5人日×40,000 ＋ Phase2 95.5人日×27,500</t>
+          <t>Phase1 35.0人日×40,000 ＋ Phase2 116.0人日×27,500</t>
         </is>
       </c>
     </row>
@@ -929,14 +929,14 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>マスタ棚卸・判定（必須）</t>
+          <t>マスタ判定後の確認（必須）</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D19" s="24" t="n">
-        <v>1600000</v>
+        <v>1080000</v>
       </c>
       <c r="E19" s="25" t="inlineStr">
         <is>
@@ -952,18 +952,18 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>マスタIF本体（仮置き）</t>
+          <t>マスタIF本体</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>95</v>
+        <v>34</v>
       </c>
       <c r="D20" s="24" t="n">
-        <v>2612500</v>
+        <v>935000</v>
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
-          <t>Phase2直接×27,500／仮置き：5本×17＋予備</t>
+          <t>Phase2直接×27,500／流用覆り：新規マスタ2本×17</t>
         </is>
       </c>
     </row>
@@ -979,10 +979,10 @@
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="D21" s="24" t="n">
-        <v>1237500</v>
+        <v>550000</v>
       </c>
       <c r="E21" s="25" t="inlineStr">
         <is>
@@ -998,10 +998,10 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>300</v>
+        <v>232</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>9056250</v>
+        <v>7155000</v>
       </c>
       <c r="E22" s="29" t="inlineStr">
         <is>
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D23" s="24" t="n">
-        <v>1200000</v>
+        <v>920000</v>
       </c>
       <c r="E23" s="25" t="inlineStr">
         <is>
@@ -1040,10 +1040,10 @@
         </is>
       </c>
       <c r="C24" s="27" t="n">
-        <v>330</v>
+        <v>255</v>
       </c>
       <c r="D24" s="28" t="n">
-        <v>10256250</v>
+        <v>8075000</v>
       </c>
       <c r="E24" s="29" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>AのPhase1分＋B1マスタ棚卸・判定</t>
+          <t>AのPhase1分＋B1確認作業</t>
         </is>
       </c>
       <c r="D28" s="30" t="n"/>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>直接工数 × (50÷499.5) ≒ 30人日</t>
+          <t>直接工数 × (50÷499.5) ≒ 23人日</t>
         </is>
       </c>
       <c r="D30" s="30" t="n"/>
@@ -1135,7 +1135,7 @@
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>4. 見積前提（不確実性含む・必読）</t>
+          <t>4. 見積前提（判定済みと残件・必読）</t>
         </is>
       </c>
       <c r="B32" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t>・【本件の性質】生鮮は調査未完の領域が多い。本提示値は「現時点の前提が成り立つ場合」の工数であり、確定請負額ではない。</t>
+          <t>・【本件の性質】2026-09-29マスタデータの判定を織り込んだ提示値。確定請負額ではない。判定が覆れば再見積。</t>
         </is>
       </c>
       <c r="B33" s="32" t="n"/>
@@ -1157,7 +1157,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
-          <t>・【最大の不確実性】生鮮専用マスタの種類・本数・非生鮮変換流用可否が未確定。影響は先行4本に閉じず PMI課題 Sinops非生鮮のPhase2（既存Sinops）全体に及ぶ。</t>
+          <t>・【判定の要点】店舗系12本は流用。勧告は2ファイルだが1.5本換算。発注統合向け変換（S26）は新規（現行生鮮→統合IFは流用不可）。入荷・スケジュールは差分。倉庫は対象外。</t>
         </is>
       </c>
       <c r="B34" s="32" t="n"/>
@@ -1168,7 +1168,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="33" t="inlineStr">
         <is>
-          <t>・【本ファイルの置き方】B1＝判定必須（Aと並行）。B2＝マスタIF仮置き。B3＝非生鮮Phase2（PMI課題）への波及バッファ。B1判定後にB2を確定値へ置換し、超過時は再見積。</t>
+          <t>・【本ファイルの置き方】A＝確定した新規／差分IF。B1＝流用突合と残件。B2＝マスタ本体IFは0。B3＝軽微波及。倉庫商品マスタ（水煮相当）は残件。</t>
         </is>
       </c>
       <c r="B35" s="34" t="n"/>
@@ -1179,7 +1179,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="33" t="inlineStr">
         <is>
-          <t>・【本案が前提とする状況】生鮮専用マスタの新規本数・既存波及が大きい場合の工数。</t>
+          <t>・【本案が前提とする状況】流用判定が一部覆る、倉庫商品マスタが要IF、またはS12/S13のSQL／作成時刻が想定より重い場合。</t>
         </is>
       </c>
       <c r="B36" s="34" t="n"/>
@@ -1190,7 +1190,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="33" t="inlineStr">
         <is>
-          <t>・【未確定の設計】勧告の連携先経路、棚割（SM/新）、営業在庫の生鮮適用、TM商品・停止・新商品在庫15等。詳細は「見積前提条件・注記」シート。</t>
+          <t>・【残る不確実性】水煮相当の倉庫商品マスタ、GCS実作業量、伝票区分・振替の項目精査、S26と発注IFの項目差、S12/S13のSQL接続と生鮮データ作成時刻。本数未確定ではない。詳細は「見積前提条件・注記」。</t>
         </is>
       </c>
       <c r="B37" s="34" t="n"/>
@@ -1255,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -1268,7 +1268,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>見積前提条件・注記（生鮮IF増分 リスク込み案 Rev.e）</t>
+          <t>見積前提条件・注記（生鮮IF増分 リスク込み案 Rev.i）</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1279,7 +1279,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="35" t="inlineStr">
         <is>
-          <t>【必読】生鮮は不確実性が大きい。下表の前提が崩れた場合、提示人日・金額は再見積対象となる。</t>
+          <t>【必読】マスタデータの流用／新規の本数は2026-09-29に判定済み。提示値は確定請負ではない。残件・覆りが顕在化したら再見積。</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -1298,31 +1298,31 @@
       <c r="D3" s="32" t="n"/>
       <c r="E3" s="32" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="37" t="inlineStr">
         <is>
-          <t>1. 本ファイルは【リスク込み案】の独立見積。調査未完の前提を置いたうえでの提示値であり、確定請負額ではない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
+          <t>1. 本ファイルは【リスク込み案】の独立見積。2026-09-29マスタデータの判定を織り込んだ提示値であり、確定請負額ではない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" s="37" t="inlineStr">
         <is>
-          <t>2. 生鮮領域は「PMI課題 Sinops非生鮮のPhase2」と同じ確度では見積もることができない。不確実性を前提に織り込んでいる。</t>
+          <t>2. 判定が覆る場合（流用→差分／新規、倉庫商品マスタが要IF）は再見積とする。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="37" t="inlineStr">
         <is>
-          <t>3. B1（マスタ棚卸・判定）完了前にB2本数は確定しない。B2は仮置き。判定後に置換し、超過時は再見積する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
+          <t>3. B2のマスタ本体IFは標準案では0。差分はAの入荷・スケジュールに計上する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
       <c r="A7" s="37" t="inlineStr">
         <is>
-          <t>4. 本案の前提状況：生鮮専用マスタの新規本数・既存波及が大きい場合の工数。</t>
+          <t>4. 本案の前提状況：流用判定が一部覆る、倉庫商品マスタが要IF、またはS12/S13のSQL／作成時刻が想定より重い場合。</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="37" t="inlineStr">
         <is>
-          <t>3. Phase1単価の対象：AのPhase1（調査用表・①②③）＋B1マスタ棚卸・判定。</t>
+          <t>3. Phase1単価の対象：AのPhase1（調査用表・①②③）＋B1流用突合・残件。</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>■ 2. 生鮮の不確実性（見積前提として明示）</t>
+          <t>■ 2. 判定済みと、残っている不確実性</t>
         </is>
       </c>
       <c r="B17" s="32" t="n"/>
@@ -1390,66 +1390,66 @@
       <c r="D17" s="32" t="n"/>
       <c r="E17" s="32" t="n"/>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="20" customHeight="1">
       <c r="A18" s="37" t="inlineStr">
         <is>
-          <t>【マスタ】生鮮は専用マスタを多数持つ。非生鮮の③変換ルールで足りるか／何本新規かは未確定。</t>
+          <t>【判定済み・流用】商品／店別／カテゴリ／仕入先／ケースバラ／POS／時間帯／来客／廃棄／在庫修正／棚割14／新商品在庫15。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="37" t="inlineStr">
         <is>
-          <t>【横断影響】マスタ前提が変わると PMI課題 Sinops非生鮮のPhase2（Sinops-01〜25）の設計・Mapping・単体にも波及し得る。</t>
+          <t>【判定済み・新規】発注勧告は当日・翌日の2ファイルだが、類似のため1.5本換算（S24=1、S25=0.5）。加えて発注統合向け変換（S26）。現行の生鮮→発注統合IFは流用不可。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="37" t="inlineStr">
         <is>
-          <t>【源・GCS】マスタ源は生鮮側サーバー→GCS。GCSに既に無ければアップロード作業が必要（会議見込：無い）。本見積に確認・アップロード作業を含む。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
+          <t>【判定済み・差分】入荷実績＝ベンダー流用、伝票区分差分、PC/CKは振替。入荷予定（nyuka_yotei）・発注スケジュール（sii.txt）＝ベンダー流用。PC/CKの生鮮データは別SQLサーバにあり、Layer①でDBGETする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
       <c r="A21" s="37" t="inlineStr">
         <is>
-          <t>【判定方法】変換ルールを1本ずつ「流用／差分／新規」の三択で判定する（B1）。一括流用は前提にしない。波多野確認：マスタの違いがあるので各IFのマッピングから始める必要がある。</t>
+          <t>【対象外】倉庫マスタ・休日・発注曜日・発注実績・受払・倉庫勧告。DC在庫なし。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="37" t="inlineStr">
         <is>
-          <t>【候補例・未確定】TM商品、店舗商品差分、カテゴリ／仕入先、停止フラグ、発注スケジュール、棚割14、新商品在庫15 等。</t>
+          <t>【残件】倉庫商品マスタ（TRIAL青果水煮相当）。要IFなら再見積。</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="37" t="inlineStr">
         <is>
-          <t>【棚割】Store Manager継続 vs 新棚割は未確定。ダミー棚の入り方により14の生鮮対応が分岐する。</t>
+          <t>【横断影響】流用前提が覆ると非生鮮Phase2にも波及し得る。契約額は据え置き。手戻りはB3。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="37" t="inlineStr">
         <is>
-          <t>【在庫】営業在庫を生鮮で使えるかは未検証。06–10系の前提再確認が必要になり得る。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
+          <t>【源・GCS】マスタ源は生鮮側サーバー→GCS。本見積に確認・必要時アップロードを含む。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="37" t="inlineStr">
         <is>
-          <t>【勧告の連携先】生鮮発注統合への直送か、自動発注GCS経由かは未確定。連携先変更はLayer①工数に効く。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
+          <t>【S12/S13の取得】TRIAL生鮮のPCとCKは別SQL。ファイル待ちではなくDBGETを各系統で置く。作成時刻はやや不安定なため、標準案のLayer①に待ち合わせを含む。日次で大きくずれる場合は再見積。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="37" t="inlineStr">
         <is>
-          <t>【入荷】入荷実績は2系統ソース（生鮮基幹＋MD基幹）、入荷予定は生鮮基幹の新規ソース。非生鮮11/12の単純流用は不可。</t>
+          <t>【Mapping難易度】高5／中4／低3。S24・S26・入荷予定・スケジュール＝高5、S25＝0.5本（2.5人日）、入荷実績＝中4。</t>
         </is>
       </c>
     </row>
@@ -1474,21 +1474,21 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="37" t="inlineStr">
         <is>
-          <t>1. A（先行トラン4本）は会議で骨格確定した新規IF。残リスクは項目精査・合流・連携先の細部。</t>
+          <t>1. A＝発注勧告2ファイルを1.5本換算＋発注統合変換1本＋入荷実績・入荷予定・発注スケジュール（差分）。</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="37" t="inlineStr">
         <is>
-          <t>2. B1＝判定そのもの（必須・AのPhase1と並行）。各IFのマッピングから着手（マスタ差分があるため）。</t>
+          <t>2. Mappingは難易度別（高5／中4／低3）。内訳（調査用表・①②③）は未分解。</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="37" t="inlineStr">
         <is>
-          <t>3. B2＝マスタIF本体の仮置き（仮置き：5本×17＋予備）。B1後に行分解して確定値へ置換。</t>
+          <t>3. B2＝流用覆り：新規マスタ2本×17。</t>
         </is>
       </c>
     </row>
@@ -1499,10 +1499,10 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
+    <row r="34" ht="20" customHeight="1">
       <c r="A34" s="37" t="inlineStr">
         <is>
-          <t>5. 仮置き超過・連携先変更・棚割方針確定などで前提が崩れた場合は増分再見積とする。</t>
+          <t>5. 再見積にするのは、流用判定の覆り、水煮相当が要IF、S26のレイアウトが非生鮮発注IFから大きく外れる、GCSが想定より重い、S12/S13のSQL接続が想定より重い、生鮮データの作成時刻が待ち合わせでは収まらない、とき。棚割は流用済み。</t>
         </is>
       </c>
     </row>
@@ -1538,10 +1538,10 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
+    <row r="40" ht="20" customHeight="1">
       <c r="A40" s="37" t="inlineStr">
         <is>
-          <t>4. PJ管理＝プロジェクト管理。GCS＝Google Cloud Storage。IF＝インターフェース。</t>
+          <t>4. PJ管理＝プロジェクト管理。GCS＝Google Cloud Storage。IF＝インターフェース。DBGET＝SQLサーバからデータを取得する処理。</t>
         </is>
       </c>
     </row>
@@ -1559,21 +1559,21 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="37" t="inlineStr">
         <is>
-          <t>1. Phase1=64.5人日（2,580,000円）＋Phase2直接=235.5人日（6,476,250円）＝直接300.0人日（9,056,250円）。</t>
+          <t>1. Phase1=62.0人日（2,480,000円）＋Phase2直接=170.0人日（4,675,000円）＝直接232.0人日（7,155,000円）。</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="37" t="inlineStr">
         <is>
-          <t>2. ＋PJ管理=30人日（1,200,000円）＝合計330.0人日／10,256,250円。</t>
+          <t>2. ＋PJ管理=23人日（920,000円）＝合計255.0人日／8,075,000円。</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="37" t="inlineStr">
         <is>
-          <t>3. 内訳 A=120.0（Phase1 24.5+Phase2 95.5）＋B1=40.0＋B2=95.0＋B3=45.0。</t>
+          <t>3. 内訳 A=151.0（Phase1 35.0+Phase2 116.0）＋B1=27.0＋B2=34.0＋B3=20.0。</t>
         </is>
       </c>
     </row>
@@ -1630,8 +1630,15 @@
         </is>
       </c>
     </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="37" t="inlineStr">
+        <is>
+          <t>6. 倉庫系IF（DC在庫なし）。倉庫商品マスタ残件が要IFとなった場合は増分再見積。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="48">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
@@ -1645,6 +1652,7 @@
     <mergeCell ref="A45:E45"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A37:E37"/>
@@ -1692,7 +1700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1708,7 +1716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【A】先行トラン4本 — Phase1＋Phase2（IF別明細／本ファイルA=120.0）</t>
+          <t>【A】確定IF — Phase1＋Phase2（IF別明細／本ファイルA=151.0）</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1722,7 +1730,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>単位：人日。本見積ファイルのAブロック値は 120.0（リスク込み案）。略語：Phase1＝調査・Mapping、Layer①＝TRIAL↔GCS、Layer②＝GCS→DWH、Layer③＝DWH・GCS↔業務。</t>
+          <t>単位：人日。本見積ファイルのAブロック値は 151.0（リスク込み案）。略語：Phase1＝調査・Mapping、Layer①＝TRIAL↔GCS、Layer②＝GCS→DWH、Layer③＝DWH・GCS↔業務。 Mapping難易度は高5／中4／低3。判定後の対象別に置いている。</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1818,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>非生鮮24と項目・ファイルが違うため新規。連携先=生鮮発注統合前提</t>
+          <t>非生鮮24と項目・ファイルが違うため新規。連携先=生鮮発注統合</t>
         </is>
       </c>
     </row>
@@ -1826,244 +1834,240 @@
         </is>
       </c>
       <c r="C7" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="19" t="n">
-        <v>1.5</v>
-      </c>
       <c r="E7" s="19" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F7" s="19" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="H7" s="21" t="inlineStr">
         <is>
-          <t>当日とレイアウト類似。未来スロット差分</t>
+          <t>当日と類似。1.5本換算の0.5本</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>生鮮入荷実績</t>
+          <t>生鮮勧告→発注統合変換</t>
         </is>
       </c>
       <c r="B8" s="39" t="inlineStr">
         <is>
-          <t>Sinops-S11</t>
+          <t>Sinops-S26</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>2.5</v>
-      </c>
       <c r="E8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="F8" s="9" t="n">
-        <v>2</v>
-      </c>
       <c r="G8" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>2系統ソース：PC/CK=生鮮基幹、取引先=MD基幹</t>
+          <t>発注統合レイアウトが非生鮮発注IFから大きく外れる場合</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="21" t="inlineStr">
         <is>
+          <t>生鮮入荷実績</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S11</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>判定覆り：2系統ソースに戻る場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>生鮮入荷予定</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B10" s="39" t="inlineStr">
         <is>
           <t>Sinops-S12</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C10" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D10" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F10" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G10" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="21" t="inlineStr">
-        <is>
-          <t>生鮮基幹新規ソース。Layer①別作</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>判定覆り：生鮮基幹を全量新規ソースとする場合。SQL2系統も前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>生鮮発注スケジュール</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S13</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>PC/CKのSQL接続・作成時刻が想定より重い場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>小計 Phase1</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr"/>
-      <c r="C10" s="26" t="inlineStr"/>
-      <c r="D10" s="26" t="inlineStr"/>
-      <c r="E10" s="26" t="inlineStr"/>
-      <c r="F10" s="26" t="inlineStr"/>
-      <c r="G10" s="27" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H10" s="29" t="n"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr"/>
+      <c r="C12" s="26" t="inlineStr"/>
+      <c r="D12" s="26" t="inlineStr"/>
+      <c r="E12" s="26" t="inlineStr"/>
+      <c r="F12" s="26" t="inlineStr"/>
+      <c r="G12" s="27" t="n">
+        <v>35</v>
+      </c>
+      <c r="H12" s="29" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>■ Layer① TRIAL↔GCS（外部IFプログラム開発）</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>IF名称</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>仮IF No.</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>項目数</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>詳細設計</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>開発</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>単体テスト</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>小計</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>生鮮発注勧告(当日分)</t>
-        </is>
-      </c>
-      <c r="B14" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S24</t>
-        </is>
-      </c>
-      <c r="C14" s="39" t="inlineStr">
-        <is>
-          <t>TBD(≠R6)</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F14" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>基準24の14に+3：連携先が生鮮発注統合</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>生鮮発注勧告(翌日以降分)</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S25</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>TBD(≠R6)</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="F15" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="G15" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="H15" s="21" t="inlineStr">
-        <is>
-          <t>基準25の14。見積行は2本</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>生鮮入荷実績</t>
+          <t>生鮮発注勧告(当日分)</t>
         </is>
       </c>
       <c r="B16" s="39" t="inlineStr">
         <is>
-          <t>Sinops-S11</t>
+          <t>Sinops-S24</t>
         </is>
       </c>
       <c r="C16" s="39" t="inlineStr">
         <is>
-          <t>TBD(~6+合流)</t>
+          <t>TBD(≠R6)</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
@@ -2080,310 +2084,514 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>基準11の10に+7：2系統合流</t>
+          <t>基準24の14に+3：生鮮勧告レイアウト差分</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="21" t="inlineStr">
         <is>
+          <t>生鮮発注勧告(翌日以降分)</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S25</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>TBD(≠R6)</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>1.5本換算の0.5本</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>生鮮勧告→発注統合変換</t>
+        </is>
+      </c>
+      <c r="B18" s="39" t="inlineStr">
+        <is>
+          <t>Sinops-S26</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>項目差分が大きく、24相当では足りない場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>生鮮入荷実績</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S11</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>TBD(~6+合流)</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>2系統合流を戻す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>生鮮入荷予定</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B20" s="39" t="inlineStr">
         <is>
           <t>Sinops-S12</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>TBD(~8)</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="E17" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="F17" s="19" t="n">
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>TBD(SQL)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G17" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>基準12の10に+4：生鮮基幹新規</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="G20" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>DBGET2系統＋作成時刻の揺れが大きい場合の再設計</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>生鮮発注スケジュール</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S13</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>TBD(SQL)</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>DBGET2系統＋作成時刻の揺れが大きい場合の再設計</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>小計 Layer①</t>
         </is>
       </c>
-      <c r="B18" s="26" t="inlineStr"/>
-      <c r="C18" s="26" t="inlineStr"/>
-      <c r="D18" s="26" t="inlineStr"/>
-      <c r="E18" s="26" t="inlineStr"/>
-      <c r="F18" s="26" t="inlineStr"/>
-      <c r="G18" s="27" t="n">
-        <v>62</v>
-      </c>
-      <c r="H18" s="29" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr"/>
+      <c r="C22" s="26" t="inlineStr"/>
+      <c r="D22" s="26" t="inlineStr"/>
+      <c r="E22" s="26" t="inlineStr"/>
+      <c r="F22" s="26" t="inlineStr"/>
+      <c r="G22" s="27" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="H22" s="29" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>■ Layer② GCS→DWH（DataSpider取込ジョブ）＝ 0（全件）</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>■ Layer③ DWH・GCS↔業務システム（DataSpider連携ジョブ）</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>IF名称</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>仮IF No.</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>項目数</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>詳細設計</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>開発</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>単体テスト</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>小計</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>生鮮発注勧告(当日分)</t>
         </is>
       </c>
-      <c r="B24" s="39" t="inlineStr">
+      <c r="B28" s="39" t="inlineStr">
         <is>
           <t>Sinops-S24</t>
         </is>
       </c>
-      <c r="C24" s="39" t="inlineStr">
+      <c r="C28" s="39" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D28" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E28" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="F24" s="9" t="n">
+      <c r="F28" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="G24" s="9" t="n">
+      <c r="G28" s="9" t="n">
         <v>4.5</v>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>基準24の3に+1.5</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="21" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>生鮮発注勧告(翌日以降分)</t>
         </is>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Sinops-S25</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D29" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E29" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="F29" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="19" t="n">
+      <c r="G29" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H29" s="21" t="inlineStr">
+        <is>
+          <t>1.5本換算の0.5本</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>生鮮勧告→発注統合変換</t>
+        </is>
+      </c>
+      <c r="B30" s="39" t="inlineStr">
+        <is>
+          <t>Sinops-S26</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>取込が想定より重い場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>生鮮入荷実績</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S11</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="21" t="inlineStr">
-        <is>
-          <t>基準25の3を維持</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>生鮮入荷実績</t>
-        </is>
-      </c>
-      <c r="B26" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S11</t>
-        </is>
-      </c>
-      <c r="C26" s="39" t="inlineStr">
+      <c r="E31" s="19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="H31" s="21" t="inlineStr">
+        <is>
+          <t>合流後取込</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>生鮮入荷予定</t>
+        </is>
+      </c>
+      <c r="B32" s="39" t="inlineStr">
+        <is>
+          <t>Sinops-S12</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D32" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E32" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>基準11の2.5に+1.5：合流後取込</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>生鮮入荷予定</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S12</t>
-        </is>
-      </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="F32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>基準12</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>生鮮発注スケジュール</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>Sinops-S13</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D33" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E33" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="19" t="n">
+      <c r="F33" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="19" t="n">
+      <c r="G33" s="19" t="n">
         <v>2.5</v>
       </c>
-      <c r="H27" s="21" t="inlineStr">
-        <is>
-          <t>基準12の2.5を維持</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="29" t="inlineStr">
+      <c r="H33" s="21" t="inlineStr">
+        <is>
+          <t>非生鮮13相当</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>小計 Layer③</t>
         </is>
       </c>
-      <c r="B28" s="26" t="inlineStr"/>
-      <c r="C28" s="26" t="inlineStr"/>
-      <c r="D28" s="26" t="inlineStr"/>
-      <c r="E28" s="26" t="inlineStr"/>
-      <c r="F28" s="26" t="inlineStr"/>
-      <c r="G28" s="27" t="n">
-        <v>14</v>
-      </c>
-      <c r="H28" s="29" t="n"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="29" t="inlineStr">
+      <c r="B34" s="26" t="inlineStr"/>
+      <c r="C34" s="26" t="inlineStr"/>
+      <c r="D34" s="26" t="inlineStr"/>
+      <c r="E34" s="26" t="inlineStr"/>
+      <c r="F34" s="26" t="inlineStr"/>
+      <c r="G34" s="27" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H34" s="29" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>Aブロック（リスク込み案）</t>
         </is>
       </c>
-      <c r="B30" s="26" t="inlineStr"/>
-      <c r="C30" s="26" t="inlineStr"/>
-      <c r="D30" s="26" t="inlineStr"/>
-      <c r="E30" s="26" t="inlineStr"/>
-      <c r="F30" s="26" t="inlineStr"/>
-      <c r="G30" s="27" t="n">
-        <v>120</v>
-      </c>
-      <c r="H30" s="29" t="inlineStr">
-        <is>
-          <t>IF別明細合計=100.5　／　本ファイル=120.0</t>
+      <c r="B36" s="26" t="inlineStr"/>
+      <c r="C36" s="26" t="inlineStr"/>
+      <c r="D36" s="26" t="inlineStr"/>
+      <c r="E36" s="26" t="inlineStr"/>
+      <c r="F36" s="26" t="inlineStr"/>
+      <c r="G36" s="27" t="n">
+        <v>151</v>
+      </c>
+      <c r="H36" s="29" t="inlineStr">
+        <is>
+          <t>IF別明細合計=151.0</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2397,11 +2605,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
@@ -2419,7 +2627,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>生鮮専用マスタは先行トランに閉じない。非生鮮中心のSinops全体に効く。</t>
+          <t>2026-09-29判定：店舗系マスタ・実績12本は流用。本体の新規マスタIFは置かない。残るのは突合と差分IF。</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -2429,7 +2637,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>■ B1 必須作業／本ファイル=40.0</t>
+          <t>■ B1 必須作業／本ファイル=27.0</t>
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -2461,267 +2669,251 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>生鮮マスタ棚卸・一覧化</t>
+          <t>流用判定の再確認</t>
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>マスタ一覧・所在マップ</t>
+          <t>再判定表</t>
         </is>
       </c>
       <c r="D6" s="41" t="inlineStr">
         <is>
-          <t>生鮮専用マスタの種類・所在・GCS有無・Sinops参照関係を一覧化</t>
+          <t>12本の一部が差分／新規に戻る場合</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>変換ルール単位の流用判定（1本ずつ）</t>
+          <t>既存Sinops横断影響調査</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>IF別 流用/差分/新規 判定表</t>
+          <t>影響リスト</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
         <is>
-          <t>既存01–05/13–15等の③変換と突合。流用／差分／新規の三択を付ける</t>
+          <t>01–25の再設計・再単体</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>既存Sinops横断影響調査</t>
+          <t>GCSアップロード・接続</t>
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>既存01–25影響リスト・改修要否</t>
+          <t>接続確認</t>
         </is>
       </c>
       <c r="D8" s="41" t="inlineStr">
         <is>
-          <t>マスタ前提が変わる場合の01–25設計・マッピング・単体観点への波及洗い出し</t>
+          <t>想定より重い場合</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>生鮮側サーバー→GCS 上げ接続確認</t>
+          <t>倉庫商品マスタ（水煮相当）新規</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>GCS接続・上げ手順の確認結果</t>
+          <t>増分IF案</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
         <is>
-          <t>会議: GCSに既にあれば再開発不要、無い見込み。見積にアップロード作業を含める</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>判定結果のゲート資料・再見積更新</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>増分IF採番案・見積更新版</t>
-        </is>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>判定表→増分IF採番→本見積のマスタIF枠を確定値に更新</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+          <t>午後MTで要IFとなった場合の調査</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>B1 本ファイル（リスク込み案）</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
-        <v>40</v>
-      </c>
-      <c r="C11" s="26" t="inlineStr"/>
-      <c r="D11" s="29" t="inlineStr"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>■ B2 マスタIF本体（仮置き）</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="B10" s="27" t="n">
+        <v>27</v>
+      </c>
+      <c r="C10" s="26" t="inlineStr"/>
+      <c r="D10" s="29" t="inlineStr"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>■ B2 マスタIF本体</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>想定</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>人日</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>算定</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>置換条件</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>新規または大幅差分のマスタIF</t>
-        </is>
-      </c>
-      <c r="B15" s="23" t="n">
-        <v>95</v>
-      </c>
-      <c r="C15" s="25" t="inlineStr">
-        <is>
-          <t>仮置き：5本×17＋予備</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="inlineStr">
-        <is>
-          <t>B1判定後に行を分解して置換</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>候補例（未確定）</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>TM商品、店舗商品差分、カテゴリ/仕入先、停止フラグ、発注スケジュール、新商品在庫15 等</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>新規マスタIF</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>34</v>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>流用覆り：新規マスタ2本×17</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>標準案は0。覆ったら再見積</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>■ B3 非生鮮Phase2（PMI課題）への波及</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>人日</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>説明</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>既存Sinops-01〜25の手戻り</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="C20" s="25" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>既存Sinopsへの手戻り</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
         <is>
           <t>複数IF再設計・再単体。非生鮮Phase2（PMI課題）の契約額は据え置き</t>
         </is>
       </c>
-      <c r="D20" s="30" t="n"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>■ 影響が及び得る既存IF（例）</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="D19" s="30" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>■ 判定後の扱い（2026-09-29）</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>既存IF</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>なぜ効くか</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>リスク</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr"/>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>見積上の扱い</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>01–05 商品・店別・カテゴリ・仕入先・ケースバラ</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>非生鮮と同じ</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>流用。B1突合のみ</t>
+        </is>
+      </c>
+      <c r="D23" s="30" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>01/02 商品・店別</t>
+          <t>06–10 POS・時間帯・来客・廃棄・在庫修正</t>
         </is>
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>TM商品・停止・発注期間が生鮮専用の可能性</t>
+          <t>非生鮮と同じ</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>変換流用不可→別IF or 分岐</t>
+          <t>流用。B1突合のみ</t>
         </is>
       </c>
       <c r="D24" s="30" t="n"/>
@@ -2729,17 +2921,17 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>03/04 カテゴリ・仕入先</t>
+          <t>14/15 棚割・新商品在庫</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>生鮮階層・仕入先体系が別</t>
+          <t>非生鮮と同じ</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>コード体系の再マッピング</t>
+          <t>流用。B1突合のみ</t>
         </is>
       </c>
       <c r="D25" s="30" t="n"/>
@@ -2747,17 +2939,17 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>05 ケースバラ</t>
+          <t>11 入荷実績</t>
         </is>
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>生鮮は計量・パック差</t>
+          <t>ベンダー流用／伝票区分差分／PC/CK振替</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>パターン追加</t>
+          <t>Aで差分IF</t>
         </is>
       </c>
       <c r="D26" s="30" t="n"/>
@@ -2765,17 +2957,17 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>13 発注スケジュール</t>
+          <t>12 入荷予定</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>生鮮締め・便・曜日が別源</t>
+          <t>ベンダー流用／PC・CKは別SQL・DBGET</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Layer①ソース分岐</t>
+          <t>Aで差分IF</t>
         </is>
       </c>
       <c r="D27" s="30" t="n"/>
@@ -2783,17 +2975,17 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>14/15 棚割・新商品在庫</t>
+          <t>13 発注スケジュール</t>
         </is>
       </c>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>生鮮は店舗調達を使わない可能性</t>
+          <t>ベンダー流用／PC・CKは別SQL・DBGET</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>15個別対応・14ダミー可否</t>
+          <t>Aで差分IF</t>
         </is>
       </c>
       <c r="D28" s="30" t="n"/>
@@ -2801,17 +2993,17 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>06–10 実績・在庫</t>
+          <t>24/25 発注勧告ファイル</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>営業在庫の生鮮適用未検証</t>
+          <t>2ファイル／1.5本換算</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>計算前提の再確認</t>
+          <t>AでS24=1本、S25=0.5本</t>
         </is>
       </c>
       <c r="D29" s="30" t="n"/>
@@ -2819,55 +3011,74 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>11/12/24/25</t>
+          <t>勧告→発注統合変換</t>
         </is>
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>先行トラン自体が新ソース</t>
+          <t>現行生鮮IFは流用不可</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>本見積Aで別計上済</t>
+          <t>Aで新規IF（S26）。参照は非生鮮24/25発注IF</t>
         </is>
       </c>
       <c r="D30" s="30" t="n"/>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="25" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>倉庫系 16–23, 倉庫勧告</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>DC在庫なし</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>対象外</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>B合計（リスク込み案）</t>
         </is>
       </c>
-      <c r="B32" s="23" t="n">
-        <v>180</v>
-      </c>
-      <c r="C32" s="25" t="inlineStr">
-        <is>
-          <t>B1 40.0 + B2 95.0 + B3 45.0</t>
-        </is>
-      </c>
-      <c r="D32" s="30" t="n"/>
+      <c r="B33" s="23" t="n">
+        <v>81</v>
+      </c>
+      <c r="C33" s="25" t="inlineStr">
+        <is>
+          <t>B1 27.0 + B2 34.0 + B3 20.0</t>
+        </is>
+      </c>
+      <c r="D33" s="30" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="A22:D22"/>
     <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C33:D33"/>
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C23:D23"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2944,17 +3155,17 @@
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>300.0 × (50/499.5) ≈ 30</t>
+          <t>232.0 × (50/499.5) ≈ 23</t>
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D5" s="28" t="n">
         <v>40000</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>1200000</v>
+        <v>920000</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -3006,7 +3217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3032,7 +3243,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>トランは新規IF必須。マスタは判定待ち（B1）。</t>
+          <t>出典: 20260929 マスタデータの判定（sinops生鮮IF.xlsx）。倉庫系はDC在庫なしで対象外。</t>
         </is>
       </c>
     </row>
@@ -3049,17 +3260,17 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>レイアウト</t>
+          <t>判定メモ</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>ソース</t>
+          <t>ソース／連携先</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>連携先</t>
+          <t>本見積</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -3071,128 +3282,288 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>生鮮勧告 当日/翌日</t>
+          <t>商品・店別・カテゴリ・仕入先・ケースバラ</t>
         </is>
       </c>
       <c r="B5" s="39" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>01–05</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>項目・ファイルが違う</t>
+          <t>非生鮮と同じ</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Sinops復路</t>
+          <t>既存</t>
         </is>
       </c>
       <c r="E5" s="39" t="inlineStr">
         <is>
-          <t>生鮮発注統合</t>
+          <t>B1突合</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>新規IF必須</t>
+          <t>流用</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>生鮮入荷実績</t>
+          <t>POS・時間帯・来客・廃棄・在庫修正</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>06–10</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>近い可能性（要精査）</t>
+          <t>非生鮮と同じ</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>生鮮基幹+MD基幹</t>
+          <t>既存</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>Sinops</t>
+          <t>B1突合</t>
         </is>
       </c>
       <c r="F6" s="21" t="inlineStr">
         <is>
-          <t>新規IF必須（2系統ソース）</t>
+          <t>流用</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>生鮮入荷予定</t>
+          <t>棚割明細・新商品在庫</t>
         </is>
       </c>
       <c r="B7" s="39" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14/15</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>近い可能性（要精査）</t>
+          <t>非生鮮と同じ</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>生鮮基幹</t>
+          <t>既存</t>
         </is>
       </c>
       <c r="E7" s="39" t="inlineStr">
         <is>
-          <t>Sinops</t>
+          <t>B1突合</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>新規IF必須</t>
+          <t>流用</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>生鮮専用マスタ群</t>
+          <t>入荷実績</t>
         </is>
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>01–05/13–15等</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>不明（大量）</t>
+          <t>伝票区分差分／PC/CKは振替</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>生鮮側サーバー</t>
+          <t>ベンダー＝既存</t>
         </is>
       </c>
       <c r="E8" s="22" t="inlineStr">
         <is>
-          <t>Sinops</t>
+          <t>A差分</t>
         </is>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>棚卸後に流用/新規判定</t>
+          <t>差分IF</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>入荷予定</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>ベンダー同じ／PC・CKは別SQL（nyuka_yotei）</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>2系統DBGET</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>A差分</t>
+        </is>
+      </c>
+      <c r="F9" s="25" t="inlineStr">
+        <is>
+          <t>差分IF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>発注スケジュール</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>ベンダー同じ／PC・CKは別SQL（sii.txt）</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>2系統DBGET</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>A差分</t>
+        </is>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>差分IF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>発注勧告 当日/翌日</t>
+        </is>
+      </c>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>24/25</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>類似のため1.5本換算</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Sinops復路</t>
+        </is>
+      </c>
+      <c r="E11" s="39" t="inlineStr">
+        <is>
+          <t>A新規</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>S24=1／S25=0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>勧告→発注統合変換</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>発注IF</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>現行生鮮→統合IFは使わない</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>非生鮮24/25参照</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>A新規</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>新規IF必須</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>倉庫マスタ・休日・実績・勧告</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>倉庫</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>DC在庫なし</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>含まない</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="inlineStr">
+        <is>
+          <t>対象外</t>
         </is>
       </c>
     </row>
@@ -3273,11 +3644,11 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>980,000円（×40,000）</t>
+          <t>1,400,000円（×40,000）</t>
         </is>
       </c>
     </row>
@@ -3293,11 +3664,11 @@
         </is>
       </c>
       <c r="C6" s="19" t="n">
-        <v>95.5</v>
+        <v>116</v>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>2,626,250円（×27,500）</t>
+          <t>3,190,000円（×27,500）</t>
         </is>
       </c>
     </row>
@@ -3309,15 +3680,15 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>IF別明細に上振れを加味</t>
+          <t>判定覆りを加味したIF別明細</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>3,606,250円</t>
+          <t>4,590,000円</t>
         </is>
       </c>
     </row>
@@ -3329,15 +3700,15 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>必須作業＋判定遅延バッファ／Phase1単価</t>
+          <t>再判定＋横断影響＋GCS＋倉庫マスタ残件／Phase1単価</t>
         </is>
       </c>
       <c r="C8" s="23" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>1,600,000円</t>
+          <t>1,080,000円</t>
         </is>
       </c>
     </row>
@@ -3349,15 +3720,15 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>仮置き：5本×17＋予備／Phase2直接</t>
+          <t>流用覆り：新規マスタ2本×17／Phase2直接</t>
         </is>
       </c>
       <c r="C9" s="23" t="n">
-        <v>95</v>
+        <v>34</v>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>2,612,500円</t>
+          <t>935,000円</t>
         </is>
       </c>
     </row>
@@ -3373,11 +3744,11 @@
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>1,237,500円</t>
+          <t>550,000円</t>
         </is>
       </c>
     </row>
@@ -3389,15 +3760,15 @@
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>Phase1 64.5+Phase2 235.5</t>
+          <t>Phase1 62.0+Phase2 170.0</t>
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>300</v>
+        <v>232</v>
       </c>
       <c r="D11" s="29" t="inlineStr">
         <is>
-          <t>9,056,250円</t>
+          <t>7,155,000円</t>
         </is>
       </c>
     </row>
@@ -3413,11 +3784,11 @@
         </is>
       </c>
       <c r="C12" s="19" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>1,200,000円（×40,000）</t>
+          <t>920,000円（×40,000）</t>
         </is>
       </c>
     </row>
@@ -3429,18 +3800,18 @@
       </c>
       <c r="B13" s="29" t="inlineStr"/>
       <c r="C13" s="27" t="n">
-        <v>330</v>
+        <v>255</v>
       </c>
       <c r="D13" s="29" t="inlineStr">
         <is>
-          <t>10,256,250円</t>
+          <t>8,075,000円</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>出典: 20260918生鮮IF会議、センター認識合わせ、既存見積Sinops明細・サマリー、単価区分は本件指定</t>
+          <t>出典: 20260929マスタデータの判定、20260918生鮮IF会議、既存見積Sinops明細・サマリー</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: align seisen increment estimate Excel, PPT, and talk tracks
Keep A/B/C labels and 仮採番 in sync, and lead briefings with premises plus 再見積 triggers instead of slogan-style risk copy.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PMI/Sinops/phase2-detail-design/sources/20260921-生鮮IF増分見積/【見積】生鮮IF増分_リスク込み案_調査Mappingから詳細設計開発単体_20260921.xlsx
+++ b/PMI/Sinops/phase2-detail-design/sources/20260921-生鮮IF増分見積/【見積】生鮮IF増分_リスク込み案_調査Mappingから詳細設計開発単体_20260921.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="サマリー" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="見積前提条件・注記" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A_先行トラン明細" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B_マスタ横断リスク" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A_新規差分IF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B_横断" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C_PJ管理" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="対既存差分" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算定根拠" sheetId="7" state="visible" r:id="rId7"/>
@@ -76,7 +76,6 @@
     </font>
     <font>
       <name val="Yu Gothic"/>
-      <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
@@ -188,6 +187,9 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -206,11 +208,14 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -218,11 +223,8 @@
     <xf numFmtId="3" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -230,20 +232,14 @@
     <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -257,12 +253,14 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -275,6 +273,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -643,20 +644,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>西友MD基幹統合　生鮮IF増分 見積（リスク込み案）</t>
+          <t>西友MD基幹統合　生鮮IF増分 見積</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -667,581 +668,505 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>見積区分</t>
+          <t>対象範囲</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>リスク込み案</t>
+          <t>調査・Mapping〜詳細設計・開発・単体（PJ管理按分を含む）</t>
         </is>
       </c>
       <c r="C2" s="5" t="n"/>
       <c r="D2" s="5" t="n"/>
       <c r="E2" s="5" t="n"/>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>作成日</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/30</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>対象範囲</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>生鮮増分のみ（Phase1調査・Mapping〜Phase2詳細設計・開発・単体テスト＋PJ管理按分）</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>非生鮮Phase2</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>PMI課題 Sinops非生鮮のPhase2。契約額は据え置き（本表は生鮮増分のみ）</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>1. 提示値（このファイルの結論）</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>1. 提示値</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>人日</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>金額（円・税抜）</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>単価</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr"/>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Phase1（調査・Mapping）</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>2480000</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>40,000</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Phase2（詳細設計・開発・単体）</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>4675000</v>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>27,500</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>PJ管理を除く</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>直接小計</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>232</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>7155000</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>A〜B3</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Phase1直接（調査・Mapping）</t>
+          <t>PJ管理</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>2480000</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>40,000 円/人日</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Phase2直接（設計・開発・単体）</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>170</v>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>4675000</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>27,500 円/人日</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>直接小計（A〜B3）</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="n">
+        <v>920000</v>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>40,000</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>直接×50/499.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>255</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>8075000</v>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>流用判定が一部覆る、倉庫商品マスタが要IF、または入荷予定・発注スケジュールのSQL／作成時刻が想定より重い場合　単価は税抜・人日（Phase1 40,000／Phase2 27,500／PJ 40,000）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>2. 内訳</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>人日</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>金額（円）</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>A（新規／差分IF）</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>勧告1.5本＋変換＋入荷2本＋スケジュール</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>151</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>4590000</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>P1 35.0／P2 116.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>B1（流用確認・残件）</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>突合、倉庫対象外、GCS、水煮残件</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>27</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>1080000</v>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Phase1単価</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>B2（マスタ本体IF）</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>店舗系マスタは流用前提</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>935000</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>流用覆り：新規マスタ2本×17</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>B3（非生鮮Phase2波及）</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>伝票区分・振替の注記</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>550000</v>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>複数IF再設計・再単体</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>直接小計</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr"/>
+      <c r="C19" s="27" t="n">
         <v>232</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="D19" s="28" t="n">
         <v>7155000</v>
       </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>混在（上表）</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>PJ管理（按分）</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n">
+      <c r="E19" s="26" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>C（PJ管理按分）</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>直接×50/499.5</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="n">
         <v>23</v>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="D20" s="22" t="n">
         <v>920000</v>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>40,000 円/人日</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>合計　【リスク込み案】</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>進捗・品質・会議</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr"/>
+      <c r="C21" s="27" t="n">
         <v>255</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="D21" s="28" t="n">
         <v>8075000</v>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　流用判定が一部覆る、倉庫商品マスタが要IF、またはS12/S13のSQL／作成時刻が想定より重い場合　／　単価：Phase1=40,000・Phase2直接=27,500・PJ管理=40,000（円/人日・税抜）</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>2. 内訳</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>ブロック</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>人日</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>金額（円）</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>内容／単価区分</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>確定IF（勧告1.5＋変換1＋入荷2＋スケジュール1）</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n">
-        <v>151</v>
-      </c>
-      <c r="D18" s="20" t="n">
-        <v>4590000</v>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
-          <t>Phase1 35.0人日×40,000 ＋ Phase2 116.0人日×27,500</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="22" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>マスタ判定後の確認（必須）</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="n">
-        <v>27</v>
-      </c>
-      <c r="D19" s="24" t="n">
-        <v>1080000</v>
-      </c>
-      <c r="E19" s="25" t="inlineStr">
-        <is>
-          <t>Phase1（調査・判定）×40,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>マスタIF本体</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="n">
-        <v>34</v>
-      </c>
-      <c r="D20" s="24" t="n">
-        <v>935000</v>
-      </c>
-      <c r="E20" s="25" t="inlineStr">
-        <is>
-          <t>Phase2直接×27,500／流用覆り：新規マスタ2本×17</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="B21" s="22" t="inlineStr">
-        <is>
-          <t>非生鮮Phase2（PMI課題）への波及</t>
-        </is>
-      </c>
-      <c r="C21" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="D21" s="24" t="n">
-        <v>550000</v>
-      </c>
-      <c r="E21" s="25" t="inlineStr">
-        <is>
-          <t>Phase2直接×27,500／複数IF再設計・再単体</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="26" t="inlineStr"/>
-      <c r="B22" s="26" t="inlineStr">
-        <is>
-          <t>直接小計</t>
-        </is>
-      </c>
-      <c r="C22" s="27" t="n">
-        <v>232</v>
-      </c>
-      <c r="D22" s="28" t="n">
-        <v>7155000</v>
-      </c>
-      <c r="E22" s="29" t="inlineStr">
-        <is>
-          <t>A＋B1＋B2＋B3</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>3. 単価</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>対象</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>単価（円/人日）</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Phase1</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>調査・Mapping、B1</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Phase2</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>27500</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>詳細設計・開発・単体（AのLayer①③、B2、B3）</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>PJ管理</t>
         </is>
       </c>
-      <c r="C23" s="23" t="n">
-        <v>23</v>
-      </c>
-      <c r="D23" s="24" t="n">
-        <v>920000</v>
-      </c>
-      <c r="E23" s="25" t="inlineStr">
-        <is>
-          <t>×40,000／進捗・品質・横断・MT（既存比率按分）</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="26" t="inlineStr"/>
-      <c r="B24" s="26" t="inlineStr">
-        <is>
-          <t>合計（リスク込み案）</t>
-        </is>
-      </c>
-      <c r="C24" s="27" t="n">
-        <v>255</v>
-      </c>
-      <c r="D24" s="28" t="n">
-        <v>8075000</v>
-      </c>
-      <c r="E24" s="29" t="inlineStr">
-        <is>
-          <t>＝ 提示値</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>3. 単価</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>対象</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>単価（円/人日）</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>備考</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr"/>
-      <c r="E27" s="8" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Phase1（調査・Mapping）</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="n">
+      <c r="B27" s="10" t="n">
         <v>40000</v>
       </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>AのPhase1分＋B1確認作業</t>
-        </is>
-      </c>
-      <c r="D28" s="30" t="n"/>
-      <c r="E28" s="30" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Phase2直接（詳細設計・開発・単体）</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="n">
-        <v>27500</v>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>AのLayer①③＋B2＋B3。PJ管理以外</t>
-        </is>
-      </c>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>PJ管理</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="n">
-        <v>40000</v>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>直接工数 × (50÷499.5) ≒ 23人日</t>
-        </is>
-      </c>
-      <c r="D30" s="30" t="n"/>
-      <c r="E30" s="30" t="n"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>4. 見積前提（判定済みと残件・必読）</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>直接 232.0 × 50/499.5 ≒ 23人日</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="29" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>4. 前提</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>・店舗系12本の流用は先方協議の結果。当社は未同席で、実データは未確認。提示は仮置きであり、確定請負ではない。</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="n"/>
+      <c r="C30" s="31" t="n"/>
+      <c r="D30" s="31" t="n"/>
+      <c r="E30" s="31" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>・勧告は2ファイルで1.5本。発注統合向け変換は新規（現行の生鮮→統合IFは使わない）。入荷・スケジュールは差分。倉庫は対象外。</t>
+        </is>
+      </c>
+      <c r="B31" s="33" t="n"/>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="33" t="n"/>
+      <c r="E31" s="33" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>・Aに新規・差分、B1に突合と残件、B2は0、B3に波及。水煮相当（倉庫商品マスタ）は残件。</t>
+        </is>
+      </c>
+      <c r="B32" s="33" t="n"/>
+      <c r="C32" s="33" t="n"/>
+      <c r="D32" s="33" t="n"/>
+      <c r="E32" s="33" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="31" t="inlineStr">
-        <is>
-          <t>・【本件の性質】2026-09-29マスタデータの判定を織り込んだ提示値。確定請負額ではない。判定が覆れば再見積。</t>
-        </is>
-      </c>
-      <c r="B33" s="32" t="n"/>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="32" t="n"/>
-      <c r="E33" s="32" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="31" t="inlineStr">
-        <is>
-          <t>・【判定の要点】店舗系12本は流用。勧告は2ファイルだが1.5本換算。発注統合向け変換（S26）は新規（現行生鮮→統合IFは流用不可）。入荷・スケジュールは差分。倉庫は対象外。</t>
-        </is>
-      </c>
-      <c r="B34" s="32" t="n"/>
-      <c r="C34" s="32" t="n"/>
-      <c r="D34" s="32" t="n"/>
-      <c r="E34" s="32" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="33" t="inlineStr">
-        <is>
-          <t>・【本ファイルの置き方】A＝確定した新規／差分IF。B1＝流用突合と残件。B2＝マスタ本体IFは0。B3＝軽微波及。倉庫商品マスタ（水煮相当）は残件。</t>
-        </is>
-      </c>
-      <c r="B35" s="34" t="n"/>
-      <c r="C35" s="34" t="n"/>
-      <c r="D35" s="34" t="n"/>
-      <c r="E35" s="34" t="n"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="33" t="inlineStr">
-        <is>
-          <t>・【本案が前提とする状況】流用判定が一部覆る、倉庫商品マスタが要IF、またはS12/S13のSQL／作成時刻が想定より重い場合。</t>
-        </is>
-      </c>
-      <c r="B36" s="34" t="n"/>
-      <c r="C36" s="34" t="n"/>
-      <c r="D36" s="34" t="n"/>
-      <c r="E36" s="34" t="n"/>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="33" t="inlineStr">
-        <is>
-          <t>・【残る不確実性】水煮相当の倉庫商品マスタ、GCS実作業量、伝票区分・振替の項目精査、S26と発注IFの項目差、S12/S13のSQL接続と生鮮データ作成時刻。本数未確定ではない。詳細は「見積前提条件・注記」。</t>
-        </is>
-      </c>
-      <c r="B37" s="34" t="n"/>
-      <c r="C37" s="34" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="34" t="n"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="33" t="inlineStr">
-        <is>
-          <t>・【動かさないもの】PMI課題 Sinops非生鮮のPhase2・共通基盤43・既存PJ管理50の契約行。結合以降・生鮮基幹本体は含まない。</t>
-        </is>
-      </c>
-      <c r="B38" s="34" t="n"/>
-      <c r="C38" s="34" t="n"/>
-      <c r="D38" s="34" t="n"/>
-      <c r="E38" s="34" t="n"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="33" t="inlineStr">
-        <is>
-          <t>・【単価】Phase1=40,000円／Phase2直接=27,500円／PJ管理=40,000円（いずれも人日・税抜）。</t>
-        </is>
-      </c>
-      <c r="B39" s="34" t="n"/>
-      <c r="C39" s="34" t="n"/>
-      <c r="D39" s="34" t="n"/>
-      <c r="E39" s="34" t="n"/>
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>・覆る場合（流用不可、水煮が要IF、SQL／作成時刻が想定外など）は再見積。非生鮮Phase2・共通基盤43・既存PJ50は動かさない。</t>
+        </is>
+      </c>
+      <c r="B33" s="33" t="n"/>
+      <c r="C33" s="33" t="n"/>
+      <c r="D33" s="33" t="n"/>
+      <c r="E33" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A34:E34"/>
+  <mergeCells count="14">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="B2:E2"/>
     <mergeCell ref="A32:E32"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="C25:E25"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1255,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -1268,7 +1193,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>見積前提条件・注記（生鮮IF増分 リスク込み案 Rev.i）</t>
+          <t>見積前提条件</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1277,416 +1202,128 @@
       <c r="E1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="35" t="inlineStr">
-        <is>
-          <t>【必読】マスタデータの流用／新規の本数は2026-09-29に判定済み。提示値は確定請負ではない。残件・覆りが顕在化したら再見積。</t>
-        </is>
-      </c>
-      <c r="B2" s="32" t="n"/>
-      <c r="C2" s="32" t="n"/>
-      <c r="D2" s="32" t="n"/>
-      <c r="E2" s="32" t="n"/>
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>店舗系12本の流用は先方協議の結果。当社は未同席。実データ未確認。確定請負ではない。</t>
+        </is>
+      </c>
+      <c r="B2" s="31" t="n"/>
+      <c r="C2" s="31" t="n"/>
+      <c r="D2" s="31" t="n"/>
+      <c r="E2" s="31" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="36" t="inlineStr">
-        <is>
-          <t>■ 0. 見積の読み方（最重要）</t>
-        </is>
-      </c>
-      <c r="B3" s="32" t="n"/>
-      <c r="C3" s="32" t="n"/>
-      <c r="D3" s="32" t="n"/>
-      <c r="E3" s="32" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="37" t="inlineStr">
-        <is>
-          <t>1. 本ファイルは【リスク込み案】の独立見積。2026-09-29マスタデータの判定を織り込んだ提示値であり、確定請負額ではない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="37" t="inlineStr">
-        <is>
-          <t>2. 判定が覆る場合（流用→差分／新規、倉庫商品マスタが要IF）は再見積とする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="37" t="inlineStr">
-        <is>
-          <t>3. B2のマスタ本体IFは標準案では0。差分はAの入荷・スケジュールに計上する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="37" t="inlineStr">
-        <is>
-          <t>4. 本案の前提状況：流用判定が一部覆る、倉庫商品マスタが要IF、またはS12/S13のSQL／作成時刻が想定より重い場合。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="38" t="inlineStr">
-        <is>
-          <t>■ 1. 範囲・契約関係・単価</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="37" t="inlineStr">
-        <is>
-          <t>1. 対象工程：Phase1（調査・Mapping）＋Phase2（詳細設計・開発・単体テスト）＋増分PJ管理按分。</t>
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>■ 範囲</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>調査・Mapping〜詳細設計・開発・単体。PJ管理按分を含む。結合以降、生鮮基幹／発注統合本体、@rms／EOS、倉庫系は含まない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>単価（税抜・人日）：Phase1 40,000円、Phase2 27,500円、PJ管理 40,000円。非生鮮Phase2・共通基盤43・既存PJ50は動かさない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>■ 流用・新規・差分</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>店舗系12本は先方協議では非生鮮と同じ。標準案はB2＝0とし、B1で突合する。覆ったら再見積。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>発注勧告は当日・翌日の2ファイル、工数は1.5本。発注統合向け変換は新規（現行の生鮮→統合IFは使わない）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>入荷実績はベンダー流用＋伝票区分差分、PC/CKは振替。入荷予定・発注スケジュールはベンダー流用、PC/CKは別SQLからDBGET。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>2. 単価：Phase1 40,000円／Phase2直接 27,500円／PJ管理 40,000円（税抜・人日）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="37" t="inlineStr">
-        <is>
-          <t>3. Phase1単価の対象：AのPhase1（調査用表・①②③）＋B1流用突合・残件。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="37" t="inlineStr">
-        <is>
-          <t>4. Phase2直接単価の対象：AのLayer①③＋B2マスタIF＋B3波及（PJ管理以外）。</t>
-        </is>
-      </c>
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>倉庫商品マスタ（水煮相当）は残件。要IFなら再見積。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>■ 数値の置き方</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="37" t="inlineStr">
-        <is>
-          <t>5. PMI課題 Sinops非生鮮のPhase2の契約額は据え置き（本表は生鮮増分のみ）。</t>
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>A 151.0人日、B1 27.0、B2 34.0、B3 20.0、直接 232.0、PJ 23、合計 255.0人日。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
-        <is>
-          <t>6. 共通基盤43・BO・既存PJ管理50の契約行も変更しない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="36" t="inlineStr">
-        <is>
-          <t>■ 2. 判定済みと、残っている不確実性</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="n"/>
-      <c r="C17" s="32" t="n"/>
-      <c r="D17" s="32" t="n"/>
-      <c r="E17" s="32" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="37" t="inlineStr">
-        <is>
-          <t>【判定済み・流用】商品／店別／カテゴリ／仕入先／ケースバラ／POS／時間帯／来客／廃棄／在庫修正／棚割14／新商品在庫15。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
-        <is>
-          <t>【判定済み・新規】発注勧告は当日・翌日の2ファイルだが、類似のため1.5本換算（S24=1、S25=0.5）。加えて発注統合向け変換（S26）。現行の生鮮→発注統合IFは流用不可。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="37" t="inlineStr">
-        <is>
-          <t>【判定済み・差分】入荷実績＝ベンダー流用、伝票区分差分、PC/CKは振替。入荷予定（nyuka_yotei）・発注スケジュール（sii.txt）＝ベンダー流用。PC/CKの生鮮データは別SQLサーバにあり、Layer①でDBGETする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="37" t="inlineStr">
-        <is>
-          <t>【対象外】倉庫マスタ・休日・発注曜日・発注実績・受払・倉庫勧告。DC在庫なし。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="37" t="inlineStr">
-        <is>
-          <t>【残件】倉庫商品マスタ（TRIAL青果水煮相当）。要IFなら再見積。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="37" t="inlineStr">
-        <is>
-          <t>【横断影響】流用前提が覆ると非生鮮Phase2にも波及し得る。契約額は据え置き。手戻りはB3。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="37" t="inlineStr">
-        <is>
-          <t>【源・GCS】マスタ源は生鮮側サーバー→GCS。本見積に確認・必要時アップロードを含む。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="37" t="inlineStr">
-        <is>
-          <t>【S12/S13の取得】TRIAL生鮮のPCとCKは別SQL。ファイル待ちではなくDBGETを各系統で置く。作成時刻はやや不安定なため、標準案のLayer①に待ち合わせを含む。日次で大きくずれる場合は再見積。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="37" t="inlineStr">
-        <is>
-          <t>【Mapping難易度】高5／中4／低3。S24・S26・入荷予定・スケジュール＝高5、S25＝0.5本（2.5人日）、入荷実績＝中4。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="37" t="inlineStr">
-        <is>
-          <t>【便】sinopsは便を持たず渡すだけ（振り分けは生鮮発注統合）。必須項目なら固定値で足りる前提。</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="38" t="inlineStr">
-        <is>
-          <t>■ 3. 本案での数値の置き方</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="37" t="inlineStr">
-        <is>
-          <t>1. A＝発注勧告2ファイルを1.5本換算＋発注統合変換1本＋入荷実績・入荷予定・発注スケジュール（差分）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
-        <is>
-          <t>2. Mappingは難易度別（高5／中4／低3）。内訳（調査用表・①②③）は未分解。</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="37" t="inlineStr">
-        <is>
-          <t>3. B2＝流用覆り：新規マスタ2本×17。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="37" t="inlineStr">
-        <is>
-          <t>4. B3＝非生鮮Phase2（PMI課題）への波及バッファ（複数IF再設計・再単体）。契約額自体は動かさない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="37" t="inlineStr">
-        <is>
-          <t>5. 再見積にするのは、流用判定の覆り、水煮相当が要IF、S26のレイアウトが非生鮮発注IFから大きく外れる、GCSが想定より重い、S12/S13のSQL接続が想定より重い、生鮮データの作成時刻が待ち合わせでは収まらない、とき。棚割は流用済み。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="38" t="inlineStr">
-        <is>
-          <t>■ 4. 略語</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="37" t="inlineStr">
-        <is>
-          <t>1. Phase1＝調査・Mapping（調査用表／①項目マッピング表／②GAP分析書／③変換ルール定義書）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="37" t="inlineStr">
-        <is>
-          <t>2. Phase2＝詳細設計・開発・単体テスト（Layer①②③の工数を含む）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="37" t="inlineStr">
-        <is>
-          <t>3. Layer①＝TRIAL↔GCS（外部IFプログラム）。Layer②＝GCS→DWH。Layer③＝DWH・GCS↔業務。</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="37" t="inlineStr">
-        <is>
-          <t>4. PJ管理＝プロジェクト管理。GCS＝Google Cloud Storage。IF＝インターフェース。DBGET＝SQLサーバからデータを取得する処理。</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="38" t="inlineStr">
-        <is>
-          <t>■ 5. 本ファイル数値</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="n"/>
-      <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="n"/>
-      <c r="E42" s="7" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="37" t="inlineStr">
-        <is>
-          <t>1. Phase1=62.0人日（2,480,000円）＋Phase2直接=170.0人日（4,675,000円）＝直接232.0人日（7,155,000円）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="37" t="inlineStr">
-        <is>
-          <t>2. ＋PJ管理=23人日（920,000円）＝合計255.0人日／8,075,000円。</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="37" t="inlineStr">
-        <is>
-          <t>3. 内訳 A=151.0（Phase1 35.0+Phase2 116.0）＋B1=27.0＋B2=34.0＋B3=20.0。</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="37" t="inlineStr">
-        <is>
-          <t>4. PJ管理按分＝直接×(50/499.5)。</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="38" t="inlineStr">
-        <is>
-          <t>■ 6. 除外（本見積に含まない）</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="37" t="inlineStr">
-        <is>
-          <t>1. 結合・総合・移行・運用テスト。</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="37" t="inlineStr">
-        <is>
-          <t>2. 生鮮基幹／生鮮発注統合本体の改修（先方）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="37" t="inlineStr">
-        <is>
-          <t>3. 青果@rms／鮮魚市場EOS等（自動補充対象外）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="37" t="inlineStr">
-        <is>
-          <t>4. 共通基盤の二重構築。</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="37" t="inlineStr">
-        <is>
-          <t>5. 店舗系非生鮮R（24/25）確定契約の読替え。</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="37" t="inlineStr">
-        <is>
-          <t>6. 倉庫系IF（DC在庫なし）。倉庫商品マスタ残件が要IFとなった場合は増分再見積。</t>
+      <c r="A15" s="36" t="inlineStr">
+        <is>
+          <t>Mappingは高5／中4／低3。Phase1小計を調査用表・①②③に分けている。S11〜S26は仮採番。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>流用が覆る、水煮が要IF、統合レイアウト差が大きい、SQL／作成時刻が想定外、のときは再見積。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A24:E24"/>
+  <mergeCells count="14">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1704,8 +1341,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -1716,7 +1353,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【A】確定IF — Phase1＋Phase2（IF別明細／本ファイルA=151.0）</t>
+          <t>A 新規・差分IF明細</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1728,9 +1365,9 @@
       <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>単位：人日。本見積ファイルのAブロック値は 151.0（リスク込み案）。略語：Phase1＝調査・Mapping、Layer①＝TRIAL↔GCS、Layer②＝GCS→DWH、Layer③＝DWH・GCS↔業務。 Mapping難易度は高5／中4／低3。判定後の対象別に置いている。</t>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>人日。Phase1は調査用表／①マッピング／②GAP／③変換ルール。S11〜S26は仮採番。 Layer①＝TRIAL↔GCS、Layer②＝GCS→DWH（本件0）、Layer③＝DWH・GCS↔業務。</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1393,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>仮IF No.</t>
+          <t>採番</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -1796,9 +1433,9 @@
           <t>生鮮発注勧告(当日分)</t>
         </is>
       </c>
-      <c r="B6" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S24</t>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>S24（仮採番）</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
@@ -1818,37 +1455,37 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>非生鮮24と項目・ファイルが違うため新規。連携先=生鮮発注統合</t>
+          <t>非生鮮発注勧告と項目・ファイルが違うため新規。連携先=生鮮発注統合</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>生鮮発注勧告(翌日以降分)</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S25</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="n">
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>S25（仮採番）</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="H7" s="20" t="inlineStr">
         <is>
           <t>当日と類似。1.5本換算の0.5本</t>
         </is>
@@ -1860,9 +1497,9 @@
           <t>生鮮勧告→発注統合変換</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S26</t>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>S26（仮採番）</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
@@ -1887,32 +1524,32 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>生鮮入荷実績</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S11</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="n">
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>S11（仮採番）</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="H9" s="20" t="inlineStr">
         <is>
           <t>判定覆り：2系統ソースに戻る場合</t>
         </is>
@@ -1924,9 +1561,9 @@
           <t>生鮮入荷予定</t>
         </is>
       </c>
-      <c r="B10" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S12</t>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>S12（仮採番）</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
@@ -1951,52 +1588,52 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>生鮮発注スケジュール</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S13</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="n">
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>S13（仮採番）</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="H11" s="21" t="inlineStr">
+      <c r="H11" s="20" t="inlineStr">
         <is>
           <t>PC/CKのSQL接続・作成時刻が想定より重い場合</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>小計 Phase1</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr"/>
-      <c r="C12" s="26" t="inlineStr"/>
-      <c r="D12" s="26" t="inlineStr"/>
-      <c r="E12" s="26" t="inlineStr"/>
-      <c r="F12" s="26" t="inlineStr"/>
+      <c r="B12" s="38" t="inlineStr"/>
+      <c r="C12" s="38" t="inlineStr"/>
+      <c r="D12" s="38" t="inlineStr"/>
+      <c r="E12" s="38" t="inlineStr"/>
+      <c r="F12" s="38" t="inlineStr"/>
       <c r="G12" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="H12" s="29" t="n"/>
+      <c r="H12" s="26" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -2020,7 +1657,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>仮IF No.</t>
+          <t>採番</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -2060,14 +1697,14 @@
           <t>生鮮発注勧告(当日分)</t>
         </is>
       </c>
-      <c r="B16" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S24</t>
-        </is>
-      </c>
-      <c r="C16" s="39" t="inlineStr">
-        <is>
-          <t>TBD(≠R6)</t>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>S24（仮採番）</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>未確定（非生鮮発注勧告は使わない）</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
@@ -2084,39 +1721,39 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>基準24の14に+3：生鮮勧告レイアウト差分</t>
+          <t>非生鮮発注勧告 Layer①14人日に+3：生鮮勧告レイアウト差分</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>生鮮発注勧告(翌日以降分)</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S25</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>TBD(≠R6)</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="n">
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>S25（仮採番）</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>未確定（非生鮮発注勧告は使わない）</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="19" t="n">
+      <c r="F17" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="G17" s="19" t="n">
+      <c r="G17" s="21" t="n">
         <v>8.5</v>
       </c>
-      <c r="H17" s="21" t="inlineStr">
+      <c r="H17" s="20" t="inlineStr">
         <is>
           <t>1.5本換算の0.5本</t>
         </is>
@@ -2128,14 +1765,14 @@
           <t>生鮮勧告→発注統合変換</t>
         </is>
       </c>
-      <c r="B18" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S26</t>
-        </is>
-      </c>
-      <c r="C18" s="39" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>S26（仮採番）</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>未確定（発注IF差が大きい場合）</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
@@ -2152,39 +1789,39 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>項目差分が大きく、24相当では足りない場合</t>
+          <t>項目差分が大きく、非生鮮発注勧告相当では足りない場合</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>生鮮入荷実績</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S11</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>TBD(~6+合流)</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="n">
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>S11（仮採番）</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>未確定（2系統合流）</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="19" t="n">
+      <c r="F19" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="19" t="n">
+      <c r="G19" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="H19" s="20" t="inlineStr">
         <is>
           <t>2系統合流を戻す</t>
         </is>
@@ -2196,14 +1833,14 @@
           <t>生鮮入荷予定</t>
         </is>
       </c>
-      <c r="B20" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S12</t>
-        </is>
-      </c>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>TBD(SQL)</t>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>S12（仮採番）</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>未確定（SQL取得）</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
@@ -2225,54 +1862,54 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>生鮮発注スケジュール</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S13</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>TBD(SQL)</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="n">
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>S13（仮採番）</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>未確定（SQL取得）</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="F21" s="19" t="n">
+      <c r="F21" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="19" t="n">
+      <c r="G21" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="H21" s="20" t="inlineStr">
         <is>
           <t>DBGET2系統＋作成時刻の揺れが大きい場合の再設計</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>小計 Layer①</t>
         </is>
       </c>
-      <c r="B22" s="26" t="inlineStr"/>
-      <c r="C22" s="26" t="inlineStr"/>
-      <c r="D22" s="26" t="inlineStr"/>
-      <c r="E22" s="26" t="inlineStr"/>
-      <c r="F22" s="26" t="inlineStr"/>
+      <c r="B22" s="38" t="inlineStr"/>
+      <c r="C22" s="38" t="inlineStr"/>
+      <c r="D22" s="38" t="inlineStr"/>
+      <c r="E22" s="38" t="inlineStr"/>
+      <c r="F22" s="38" t="inlineStr"/>
       <c r="G22" s="27" t="n">
         <v>95.5</v>
       </c>
-      <c r="H22" s="29" t="n"/>
+      <c r="H22" s="26" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -2310,7 +1947,7 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>仮IF No.</t>
+          <t>採番</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -2350,14 +1987,14 @@
           <t>生鮮発注勧告(当日分)</t>
         </is>
       </c>
-      <c r="B28" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S24</t>
-        </is>
-      </c>
-      <c r="C28" s="39" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>S24（仮採番）</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>未確定</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
@@ -2374,39 +2011,39 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>基準24の3に+1.5</t>
+          <t>非生鮮発注勧告 Layer③3人日に+1.5</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>生鮮発注勧告(翌日以降分)</t>
         </is>
       </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S25</t>
-        </is>
-      </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D29" s="19" t="n">
+      <c r="B29" s="37" t="inlineStr">
+        <is>
+          <t>S25（仮採番）</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>未確定</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E29" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="19" t="n">
+      <c r="F29" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="19" t="n">
+      <c r="G29" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="H29" s="21" t="inlineStr">
+      <c r="H29" s="20" t="inlineStr">
         <is>
           <t>1.5本換算の0.5本</t>
         </is>
@@ -2418,14 +2055,14 @@
           <t>生鮮勧告→発注統合変換</t>
         </is>
       </c>
-      <c r="B30" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S26</t>
-        </is>
-      </c>
-      <c r="C30" s="39" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>S26（仮採番）</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>未確定</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
@@ -2447,34 +2084,34 @@
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>生鮮入荷実績</t>
         </is>
       </c>
-      <c r="B31" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S11</t>
-        </is>
-      </c>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="n">
+      <c r="B31" s="37" t="inlineStr">
+        <is>
+          <t>S11（仮採番）</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>未確定</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="F31" s="19" t="n">
+      <c r="F31" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="G31" s="19" t="n">
+      <c r="G31" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H31" s="21" t="inlineStr">
+      <c r="H31" s="20" t="inlineStr">
         <is>
           <t>合流後取込</t>
         </is>
@@ -2486,14 +2123,14 @@
           <t>生鮮入荷予定</t>
         </is>
       </c>
-      <c r="B32" s="39" t="inlineStr">
-        <is>
-          <t>Sinops-S12</t>
-        </is>
-      </c>
-      <c r="C32" s="39" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>S12（仮採番）</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>未確定</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
@@ -2510,79 +2147,75 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>基準12</t>
+          <t>非生鮮入荷予定 Layer③相当</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>生鮮発注スケジュール</t>
         </is>
       </c>
-      <c r="B33" s="18" t="inlineStr">
-        <is>
-          <t>Sinops-S13</t>
-        </is>
-      </c>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="n">
+      <c r="B33" s="37" t="inlineStr">
+        <is>
+          <t>S13（仮採番）</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>未確定</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="E33" s="19" t="n">
+      <c r="E33" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="F33" s="19" t="n">
+      <c r="F33" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="19" t="n">
+      <c r="G33" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="H33" s="21" t="inlineStr">
-        <is>
-          <t>非生鮮13相当</t>
+      <c r="H33" s="20" t="inlineStr">
+        <is>
+          <t>非生鮮発注スケジュール相当</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="29" t="inlineStr">
+      <c r="A34" s="26" t="inlineStr">
         <is>
           <t>小計 Layer③</t>
         </is>
       </c>
-      <c r="B34" s="26" t="inlineStr"/>
-      <c r="C34" s="26" t="inlineStr"/>
-      <c r="D34" s="26" t="inlineStr"/>
-      <c r="E34" s="26" t="inlineStr"/>
-      <c r="F34" s="26" t="inlineStr"/>
+      <c r="B34" s="38" t="inlineStr"/>
+      <c r="C34" s="38" t="inlineStr"/>
+      <c r="D34" s="38" t="inlineStr"/>
+      <c r="E34" s="38" t="inlineStr"/>
+      <c r="F34" s="38" t="inlineStr"/>
       <c r="G34" s="27" t="n">
         <v>20.5</v>
       </c>
-      <c r="H34" s="29" t="n"/>
+      <c r="H34" s="26" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="29" t="inlineStr">
-        <is>
-          <t>Aブロック（リスク込み案）</t>
-        </is>
-      </c>
-      <c r="B36" s="26" t="inlineStr"/>
-      <c r="C36" s="26" t="inlineStr"/>
-      <c r="D36" s="26" t="inlineStr"/>
-      <c r="E36" s="26" t="inlineStr"/>
-      <c r="F36" s="26" t="inlineStr"/>
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>A 計</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr"/>
+      <c r="C36" s="38" t="inlineStr"/>
+      <c r="D36" s="38" t="inlineStr"/>
+      <c r="E36" s="38" t="inlineStr"/>
+      <c r="F36" s="38" t="inlineStr"/>
       <c r="G36" s="27" t="n">
         <v>151</v>
       </c>
-      <c r="H36" s="29" t="inlineStr">
-        <is>
-          <t>IF別明細合計=151.0</t>
-        </is>
-      </c>
+      <c r="H36" s="26" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2617,7 +2250,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【B】生鮮専用マスタ横断リスク（リスク込み案）</t>
+          <t>B 横断（流用確認・マスタIF・波及）</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2625,19 +2258,19 @@
       <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>2026-09-29判定：店舗系マスタ・実績12本は流用。本体の新規マスタIFは置かない。残るのは突合と差分IF。</t>
-        </is>
-      </c>
-      <c r="B2" s="32" t="n"/>
-      <c r="C2" s="32" t="n"/>
-      <c r="D2" s="32" t="n"/>
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>店舗系12本は先方協議では流用。当社未同席。本体IFは置かず、B1で突合する。</t>
+        </is>
+      </c>
+      <c r="B2" s="31" t="n"/>
+      <c r="C2" s="31" t="n"/>
+      <c r="D2" s="31" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>■ B1 必須作業／本ファイル=27.0</t>
+          <t>■ B1 流用確認・残件　27.0人日</t>
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -2667,20 +2300,20 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>流用判定の再確認</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>再判定表</t>
         </is>
       </c>
-      <c r="D6" s="41" t="inlineStr">
+      <c r="D6" s="40" t="inlineStr">
         <is>
           <t>12本の一部が差分／新規に戻る場合</t>
         </is>
@@ -2700,27 +2333,27 @@
           <t>影響リスト</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>01–25の再設計・再単体</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>GCSアップロード・接続</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>接続確認</t>
         </is>
       </c>
-      <c r="D8" s="41" t="inlineStr">
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>想定より重い場合</t>
         </is>
@@ -2740,28 +2373,28 @@
           <t>増分IF案</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>午後MTで要IFとなった場合の調査</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>B1 本ファイル（リスク込み案）</t>
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>B1 計</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="C10" s="26" t="inlineStr"/>
-      <c r="D10" s="29" t="inlineStr"/>
+      <c r="C10" s="38" t="inlineStr"/>
+      <c r="D10" s="26" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>■ B2 マスタIF本体</t>
+          <t>■ B2 マスタ本体IF</t>
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
@@ -2791,20 +2424,20 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>新規マスタIF</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="24" t="n">
         <v>34</v>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>流用覆り：新規マスタ2本×17</t>
         </is>
       </c>
-      <c r="D14" s="25" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>標準案は0。覆ったら再見積</t>
         </is>
@@ -2813,7 +2446,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>■ B3 非生鮮Phase2（PMI課題）への波及</t>
+          <t>■ B3 非生鮮Phase2波及</t>
         </is>
       </c>
       <c r="B17" s="7" t="n"/>
@@ -2839,25 +2472,25 @@
       <c r="D18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>既存Sinopsへの手戻り</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t>複数IF再設計・再単体。非生鮮Phase2（PMI課題）の契約額は据え置き</t>
-        </is>
-      </c>
-      <c r="D19" s="30" t="n"/>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>複数IF再設計・再単体。非生鮮Phase2の契約額は据え置き</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>■ 判定後の扱い（2026-09-29）</t>
+          <t>■ 判定後の扱い</t>
         </is>
       </c>
       <c r="B21" s="7" t="n"/>
@@ -2885,79 +2518,79 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>01–05 商品・店別・カテゴリ・仕入先・ケースバラ</t>
+          <t>商品・店別・カテゴリ・仕入先・ケースバラ</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>非生鮮と同じ</t>
+          <t>先方協議では非生鮮と同じ</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>流用。B1突合のみ</t>
-        </is>
-      </c>
-      <c r="D23" s="30" t="n"/>
+          <t>流用（B1で突合）</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>06–10 POS・時間帯・来客・廃棄・在庫修正</t>
-        </is>
-      </c>
-      <c r="B24" s="21" t="inlineStr">
-        <is>
-          <t>非生鮮と同じ</t>
-        </is>
-      </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>流用。B1突合のみ</t>
-        </is>
-      </c>
-      <c r="D24" s="30" t="n"/>
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>POS・時間帯・来客・廃棄・在庫修正</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>先方協議では非生鮮と同じ</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>流用（B1で突合）</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>14/15 棚割・新商品在庫</t>
+          <t>棚割・新商品在庫</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>非生鮮と同じ</t>
+          <t>先方協議では非生鮮と同じ</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>流用。B1突合のみ</t>
-        </is>
-      </c>
-      <c r="D25" s="30" t="n"/>
+          <t>流用（B1で突合）</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>11 入荷実績</t>
-        </is>
-      </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>入荷実績</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>ベンダー流用／伝票区分差分／PC/CK振替</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>Aで差分IF</t>
-        </is>
-      </c>
-      <c r="D26" s="30" t="n"/>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>A 差分</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>12 入荷予定</t>
+          <t>入荷予定</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2967,33 +2600,33 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Aで差分IF</t>
-        </is>
-      </c>
-      <c r="D27" s="30" t="n"/>
+          <t>A 差分</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>13 発注スケジュール</t>
-        </is>
-      </c>
-      <c r="B28" s="21" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>発注スケジュール</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>ベンダー流用／PC・CKは別SQL・DBGET</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>Aで差分IF</t>
-        </is>
-      </c>
-      <c r="D28" s="30" t="n"/>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>A 差分</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>24/25 発注勧告ファイル</t>
+          <t>発注勧告（当日／翌日以降）</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -3003,33 +2636,33 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>AでS24=1本、S25=0.5本</t>
-        </is>
-      </c>
-      <c r="D29" s="30" t="n"/>
+          <t>A 新規</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>勧告→発注統合変換</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
-        <is>
-          <t>現行生鮮IFは流用不可</t>
-        </is>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>Aで新規IF（S26）。参照は非生鮮24/25発注IF</t>
-        </is>
-      </c>
-      <c r="D30" s="30" t="n"/>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>現行生鮮→統合IFは使わない</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>A 新規</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>倉庫系 16–23, 倉庫勧告</t>
+          <t>倉庫マスタ・休日・実績・勧告</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -3042,23 +2675,23 @@
           <t>対象外</t>
         </is>
       </c>
-      <c r="D31" s="30" t="n"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
-        <is>
-          <t>B合計（リスク込み案）</t>
-        </is>
-      </c>
-      <c r="B33" s="23" t="n">
+      <c r="D31" s="29" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>B 計</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="n">
         <v>81</v>
       </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>B1 27.0 + B2 34.0 + B3 20.0</t>
-        </is>
-      </c>
-      <c r="D33" s="30" t="n"/>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>B1 27.0 ＋ B2 34.0 ＋ B3 20.0</t>
+        </is>
+      </c>
+      <c r="D33" s="29" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -3105,7 +2738,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【C】PJ管理（増分按分・リスク込み案）</t>
+          <t>C PJ管理按分</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3114,7 +2747,7 @@
       <c r="E1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>既存PJ管理50は開発スコープ499.5横断分。本増分は同じ比率50/499.5を本ファイル直接工数に適用。</t>
         </is>
@@ -3148,12 +2781,12 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>PJ管理（リスク込み案）</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>PJ管理</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>232.0 × (50/499.5) ≈ 23</t>
         </is>
@@ -3169,7 +2802,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t>含む作業</t>
         </is>
@@ -3179,12 +2812,12 @@
           <t>進捗・品質管理、横断課題対応、会議体（MT）対応など</t>
         </is>
       </c>
-      <c r="C7" s="30" t="n"/>
-      <c r="D7" s="30" t="n"/>
-      <c r="E7" s="30" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="29" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>既存契約</t>
         </is>
@@ -3194,9 +2827,9 @@
           <t>既存PJ管理50の契約行は変更しない。本表は生鮮増分の追加PJ管理。</t>
         </is>
       </c>
-      <c r="C8" s="30" t="n"/>
-      <c r="D8" s="30" t="n"/>
-      <c r="E8" s="30" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="29" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3221,17 +2854,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>既存IF流用可否と新規判定</t>
+          <t>流用可否</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3241,9 +2874,9 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>出典: 20260929 マスタデータの判定（sinops生鮮IF.xlsx）。倉庫系はDC在庫なしで対象外。</t>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>出典：2026-09-29 マスタデータ判定。倉庫系はDC在庫なしで対象外。</t>
         </is>
       </c>
     </row>
@@ -3285,14 +2918,14 @@
           <t>商品・店別・カテゴリ・仕入先・ケースバラ</t>
         </is>
       </c>
-      <c r="B5" s="39" t="inlineStr">
-        <is>
-          <t>01–05</t>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>非生鮮同名マスタ</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>非生鮮と同じ</t>
+          <t>先方協議では非生鮮と同じ</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -3300,46 +2933,46 @@
           <t>既存</t>
         </is>
       </c>
-      <c r="E5" s="39" t="inlineStr">
-        <is>
-          <t>B1突合</t>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>B1</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>流用</t>
+          <t>流用（未確認）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>POS・時間帯・来客・廃棄・在庫修正</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>06–10</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>非生鮮と同じ</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>非生鮮同名実績</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>先方協議では非生鮮と同じ</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>既存</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>B1突合</t>
-        </is>
-      </c>
-      <c r="F6" s="21" t="inlineStr">
-        <is>
-          <t>流用</t>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>流用（未確認）</t>
         </is>
       </c>
     </row>
@@ -3349,14 +2982,14 @@
           <t>棚割明細・新商品在庫</t>
         </is>
       </c>
-      <c r="B7" s="39" t="inlineStr">
-        <is>
-          <t>14/15</t>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>非生鮮棚割・新商品在庫</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>非生鮮と同じ</t>
+          <t>先方協議では非生鮮と同じ</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -3364,110 +2997,110 @@
           <t>既存</t>
         </is>
       </c>
-      <c r="E7" s="39" t="inlineStr">
-        <is>
-          <t>B1突合</t>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>B1</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>流用</t>
+          <t>流用（未確認）</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>入荷実績</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="inlineStr">
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>非生鮮入荷実績</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>伝票区分差分／PC/CKは振替</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>ベンダー＝既存</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
-        <is>
-          <t>A差分</t>
-        </is>
-      </c>
-      <c r="F8" s="25" t="inlineStr">
-        <is>
-          <t>差分IF</t>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>差分</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>入荷予定</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>ベンダー同じ／PC・CKは別SQL（nyuka_yotei）</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>非生鮮入荷予定</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ベンダー同じ／PC・CKは別SQL</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>2系統DBGET</t>
         </is>
       </c>
-      <c r="E9" s="22" t="inlineStr">
-        <is>
-          <t>A差分</t>
-        </is>
-      </c>
-      <c r="F9" s="25" t="inlineStr">
-        <is>
-          <t>差分IF</t>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>差分</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>発注スケジュール</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>ベンダー同じ／PC・CKは別SQL（sii.txt）</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>非生鮮発注スケジュール</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>ベンダー同じ／PC・CKは別SQL</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>2系統DBGET</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>A差分</t>
-        </is>
-      </c>
-      <c r="F10" s="25" t="inlineStr">
-        <is>
-          <t>差分IF</t>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>差分</t>
         </is>
       </c>
     </row>
@@ -3477,9 +3110,9 @@
           <t>発注勧告 当日/翌日</t>
         </is>
       </c>
-      <c r="B11" s="39" t="inlineStr">
-        <is>
-          <t>24/25</t>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>非生鮮発注勧告</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -3492,76 +3125,76 @@
           <t>Sinops復路</t>
         </is>
       </c>
-      <c r="E11" s="39" t="inlineStr">
-        <is>
-          <t>A新規</t>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>S24=1／S25=0.5</t>
+          <t>新規</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>勧告→発注統合変換</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>発注IF</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>非生鮮発注勧告</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>現行生鮮→統合IFは使わない</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
-        <is>
-          <t>非生鮮24/25参照</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>A新規</t>
-        </is>
-      </c>
-      <c r="F12" s="21" t="inlineStr">
-        <is>
-          <t>新規IF必須</t>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>非生鮮発注勧告を参照</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>新規</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>倉庫マスタ・休日・実績・勧告</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="43" t="inlineStr">
         <is>
           <t>倉庫</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>DC在庫なし</t>
         </is>
       </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="22" t="inlineStr">
-        <is>
-          <t>含まない</t>
-        </is>
-      </c>
-      <c r="F13" s="25" t="inlineStr">
+      <c r="E13" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>対象外</t>
         </is>
@@ -3587,7 +3220,7 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
@@ -3596,7 +3229,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>算定根拠（リスク込み案）</t>
+          <t>算定根拠</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3604,9 +3237,9 @@
       <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>本ファイルは【リスク込み案】の独立見積。単価：Phase1=40,000／Phase2直接=27,500／PJ=40,000。</t>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>単価：Phase1 40,000／Phase2 27,500／PJ 40,000（円・人日・税抜）。</t>
         </is>
       </c>
     </row>
@@ -3618,7 +3251,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>基準/仮定</t>
+          <t>内容</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -3628,7 +3261,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>金額・根拠</t>
+          <t>金額</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3273,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>調査・Mapping明細</t>
+          <t>調査・Mapping</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
@@ -3648,34 +3281,34 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1,400,000円（×40,000）</t>
+          <t>1,400,000</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>A Phase2</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Layer①③（Layer②=0）</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="n">
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Layer①③</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="n">
         <v>116</v>
       </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>3,190,000円（×27,500）</t>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>3,190,000</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>A 小計</t>
+          <t>A 計</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -3688,128 +3321,128 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>4,590,000円</t>
+          <t>4,590,000</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>B1 必須</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>再判定＋横断影響＋GCS＋倉庫マスタ残件／Phase1単価</t>
-        </is>
-      </c>
-      <c r="C8" s="23" t="n">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>再判定＋横断影響＋GCS＋倉庫マスタ残件</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n">
         <v>27</v>
       </c>
-      <c r="D8" s="25" t="inlineStr">
-        <is>
-          <t>1,080,000円</t>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>1,080,000</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>B2 マスタIF</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
-        <is>
-          <t>流用覆り：新規マスタ2本×17／Phase2直接</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="n">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>流用覆り：新規マスタ2本×17</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="n">
         <v>34</v>
       </c>
-      <c r="D9" s="25" t="inlineStr">
-        <is>
-          <t>935,000円</t>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>935,000</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>B3 非生鮮Phase2波及</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="inlineStr">
-        <is>
-          <t>複数IF再設計・再単体／Phase2直接</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="n">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>複数IF再設計・再単体</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="D10" s="25" t="inlineStr">
-        <is>
-          <t>550,000円</t>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>550,000</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>直接小計</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Phase1 62.0+Phase2 170.0</t>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Phase1 62.0＋Phase2 170.0</t>
         </is>
       </c>
       <c r="C11" s="27" t="n">
         <v>232</v>
       </c>
-      <c r="D11" s="29" t="inlineStr">
-        <is>
-          <t>7,155,000円</t>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>7,155,000</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>C PJ管理</t>
-        </is>
-      </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>50/499.5 按分</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="n">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>C PJ</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>50/499.5</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="n">
         <v>23</v>
       </c>
-      <c r="D12" s="21" t="inlineStr">
-        <is>
-          <t>920,000円（×40,000）</t>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>920,000</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>合計（リスク込み案）</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr"/>
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr"/>
       <c r="C13" s="27" t="n">
         <v>255</v>
       </c>
-      <c r="D13" s="29" t="inlineStr">
-        <is>
-          <t>8,075,000円</t>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>8,075,000</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>出典: 20260929マスタデータの判定、20260918生鮮IF会議、既存見積Sinops明細・サマリー</t>
         </is>

</xml_diff>